<commit_message>
📊 Horarios actualizados Línea 141 - 4356
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:28:55</t>
+          <t>Última actualización: 01:10:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:28:55</t>
+          <t>01:10:53</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -487,9 +487,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>01:10:53</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>03:01</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>111</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -519,7 +544,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:28:55</t>
+          <t>Última actualización: 01:10:53</t>
         </is>
       </c>
     </row>
@@ -554,7 +579,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:28:55</t>
+          <t>Última actualización: 01:10:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4357
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:10:53</t>
+          <t>Última actualización: 01:58:15</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:10:53</t>
+          <t>01:58:15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:25</t>
+          <t>03:02</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>64</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:10:53</t>
+          <t>01:58:15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:01</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:10:53</t>
+          <t>Última actualización: 01:58:15</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:10:53</t>
+          <t>Última actualización: 01:58:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4358
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:58:15</t>
+          <t>Última actualización: 02:30:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:58:15</t>
+          <t>02:30:58</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>64</v>
+        <v>31</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,12 +498,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:58:15</t>
+          <t>02:30:58</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>03:47</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -512,9 +512,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>110</v>
+        <v>77</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:30:58</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>91</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -544,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:58:15</t>
+          <t>Última actualización: 02:30:58</t>
         </is>
       </c>
     </row>
@@ -579,7 +604,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:58:15</t>
+          <t>Última actualización: 02:30:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4359
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:30:58</t>
+          <t>Última actualización: 03:02:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:30:58</t>
+          <t>03:02:42</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:01</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:30:58</t>
+          <t>03:02:42</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:47</t>
+          <t>04:02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,23 +523,73 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:30:58</t>
+          <t>03:02:42</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:01</t>
+          <t>04:29</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:02:42</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:47</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>91</v>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D9" t="n">
+        <v>105</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>03:02:42</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>04:53</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>111</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -569,7 +619,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:30:58</t>
+          <t>Última actualización: 03:02:42</t>
         </is>
       </c>
     </row>
@@ -604,7 +654,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:30:58</t>
+          <t>Última actualización: 03:02:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4360
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:02:42</t>
+          <t>Última actualización: 04:10:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:02:42</t>
+          <t>04:10:52</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:02:42</t>
+          <t>04:10:52</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:02:42</t>
+          <t>04:10:52</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:29</t>
+          <t>05:16</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:02:42</t>
+          <t>04:10:52</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>05:21</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,23 +573,98 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:02:42</t>
+          <t>04:10:52</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:43</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>04:10:52</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:46</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>96</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04:10:52</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>110</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:10:52</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:08</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>118</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -619,7 +694,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:02:42</t>
+          <t>Última actualización: 04:10:52</t>
         </is>
       </c>
     </row>
@@ -654,7 +729,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:02:42</t>
+          <t>Última actualización: 04:10:52</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4361
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:10:52</t>
+          <t>Última actualización: 05:00:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:10:52</t>
+          <t>05:00:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>05:01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:10:52</t>
+          <t>05:00:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:10:52</t>
+          <t>05:00:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:16</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:10:52</t>
+          <t>05:00:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:21</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:10:52</t>
+          <t>05:00:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:43</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>93</v>
+        <v>61</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:10:52</t>
+          <t>05:00:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:46</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:10:52</t>
+          <t>05:00:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>110</v>
+        <v>72</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,23 +648,173 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:10:52</t>
+          <t>05:00:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:08</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>118</v>
+        <v>90</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>05:00:30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:36</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>96</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>05:00:30</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>99</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>05:00:30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>101</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>05:00:30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>101</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>05:00:30</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:44</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>104</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>05:00:30</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>06:59</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>119</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -681,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -694,14 +844,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:10:52</t>
+          <t>Última actualización: 05:00:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>05:00:30</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>72</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -729,7 +931,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:10:52</t>
+          <t>Última actualización: 05:00:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4362
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:00:30</t>
+          <t>Última actualización: 05:54:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:01</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>90</v>
+        <v>47</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>99</v>
+        <v>68</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:44</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,23 +798,48 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>05:54:40</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>110</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -831,7 +856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -844,14 +869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:00:30</t>
+          <t>Última actualización: 05:54:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -885,7 +910,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:00:30</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -899,9 +924,59 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:54:40</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>68</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05:54:40</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>97</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -918,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -931,14 +1006,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:00:30</t>
+          <t>Última actualización: 05:54:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>05:54:40</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>114</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4363
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:54:40</t>
+          <t>Última actualización: 06:28:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>06:28:10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>06:28:10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>06:28:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>06:28:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -658,11 +658,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>06:28:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>06:28:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>06:46</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>06:28:10</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>93</v>
+        <v>31</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>06:28:10</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>06:28:10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>06:28:10</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -828,18 +828,268 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>97</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>05:54:40</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>97</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06:28:10</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>64</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>05:54:40</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>102</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>06:28:10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>69</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>06:28:10</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>07:44</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>110</v>
-      </c>
-      <c r="E20" t="inlineStr">
+      <c r="D25" t="n">
+        <v>76</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>06:28:10</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>83</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>06:28:10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>07:59</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>91</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>06:28:10</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>93</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>06:28:10</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>111</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>06:28:10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>118</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -856,7 +1106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -869,14 +1119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:54:40</t>
+          <t>Última actualización: 06:28:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -935,7 +1185,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>06:28:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -949,7 +1199,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -977,6 +1227,56 @@
         <v>97</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:28:10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>64</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:28:10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>83</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -993,7 +1293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1006,14 +1306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:54:40</t>
+          <t>Última actualización: 06:28:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -1064,6 +1364,31 @@
         <v>114</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06:28:10</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>81</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4364
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:28:10</t>
+          <t>Última actualización: 07:03:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:28:10</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:03</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:28:10</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:04</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>97</v>
+        <v>24</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>06:28:10</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>97</v>
+        <v>60</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:28:10</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>102</v>
+        <v>28</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,21 +923,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>06:28:10</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -953,16 +953,16 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:28:10</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>83</v>
+        <v>33</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:28:10</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>93</v>
+        <v>41</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>06:28:10</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>111</v>
+        <v>48</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1078,18 +1078,243 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>07:59</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>91</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>58</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>08:06</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>63</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>76</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>78</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>82</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>06:28:10</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>08:26</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D36" t="n">
         <v>118</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>08:35</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>92</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>101</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>101</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1106,7 +1331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1119,14 +1344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:28:10</t>
+          <t>Última actualización: 07:03:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1210,21 +1435,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:03</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1235,12 +1460,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06:28:10</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1249,7 +1474,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1265,18 +1490,93 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>64</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>07:51</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>83</v>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="D11" t="n">
+        <v>48</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>101</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>101</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1293,7 +1593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1306,14 +1606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:28:10</t>
+          <t>Última actualización: 07:03:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1647,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1361,7 +1661,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>114</v>
+        <v>45</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1391,6 +1691,56 @@
       <c r="E7" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>94</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:03:46</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>119</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4365
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:03:46</t>
+          <t>Última actualización: 07:41:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>101</v>
+        <v>60</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,13 +1308,188 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>63</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>07:41:47</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D39" t="n">
-        <v>101</v>
-      </c>
-      <c r="E39" t="inlineStr">
+      <c r="D40" t="n">
+        <v>63</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>07:41:47</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>83</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>07:41:47</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>85</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>07:41:47</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>09:13</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>92</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>07:41:47</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>103</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>07:41:47</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>113</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>07:41:47</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>114</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1331,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1344,14 +1519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:03:46</t>
+          <t>Última actualización: 07:41:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1685,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1524,7 +1699,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1535,7 +1710,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1549,7 +1724,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>101</v>
+        <v>63</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1560,7 +1735,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1574,9 +1749,34 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>101</v>
+        <v>63</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07:41:47</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>85</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1606,7 +1806,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:03:46</t>
+          <t>Última actualización: 07:41:47</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1847,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1661,7 +1861,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1697,7 +1897,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1711,7 +1911,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1722,7 +1922,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>07:41:47</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1736,7 +1936,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>119</v>
+        <v>81</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4366
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:41:47</t>
+          <t>Última actualización: 08:02:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>83</v>
+        <v>42</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>09:13</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:13</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,23 +1473,198 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>08:02:51</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>74</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>08:02:51</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>81</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>07:41:47</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>103</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>08:02:51</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>92</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>08:02:51</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>09:35</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D46" t="n">
-        <v>114</v>
-      </c>
-      <c r="E46" t="inlineStr">
+      <c r="D50" t="n">
+        <v>93</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>08:02:51</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>102</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>08:02:51</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>112</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>08:02:51</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>116</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1506,7 +1681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1519,14 +1694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:41:47</t>
+          <t>Última actualización: 08:02:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1885,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1724,7 +1899,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1735,7 +1910,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1749,7 +1924,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1760,7 +1935,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1774,9 +1949,34 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:02:51</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>112</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1793,7 +1993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1806,14 +2006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:41:47</t>
+          <t>Última actualización: 08:02:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1897,7 +2097,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1911,7 +2111,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1922,7 +2122,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1936,11 +2136,36 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>08:02:51</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>85</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4367
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:02:51</t>
+          <t>Última actualización: 08:34:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>09:13</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>71</v>
+        <v>30</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1503,16 +1503,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>09:23</t>
+          <t>09:13</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:41:47</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>103</v>
+        <v>42</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1578,16 +1578,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:23</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>102</v>
+        <v>50</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>112</v>
+        <v>60</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,23 +1648,223 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>61</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>70</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>08:02:51</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>112</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>81</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>08:02:51</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
         <is>
           <t>09:58</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D53" t="n">
+      <c r="D57" t="n">
         <v>116</v>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>87</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>90</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>101</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>110</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1681,7 +1881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1694,14 +1894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:02:51</t>
+          <t>Última actualización: 08:34:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -1885,7 +2085,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1899,7 +2099,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1935,21 +2135,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1960,23 +2160,73 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>32</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>08:02:51</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>09:54</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D16" t="n">
         <v>112</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>81</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1993,7 +2243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2006,14 +2256,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:02:51</t>
+          <t>Última actualización: 08:34:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -2122,25 +2372,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09:02</t>
+          <t>08:38</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
@@ -2152,18 +2402,143 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>60</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>29</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>08:02:51</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>09:27</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D12" t="n">
         <v>85</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>54</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>104</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>116</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4368
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:34:29</t>
+          <t>Última actualización: 08:53:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 56</t>
+          <t>Total filas: 59</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1462,7 +1462,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,7 +1623,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,7 +1648,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1662,7 +1662,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>112</v>
+        <v>61</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1862,9 +1862,84 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>08:53:40</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>93</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>08:53:40</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>101</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>08:53:40</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>111</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1894,7 +1969,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:34:29</t>
+          <t>Última actualización: 08:53:40</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2235,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2174,7 +2249,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2185,7 +2260,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2199,7 +2274,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>112</v>
+        <v>61</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2243,7 +2318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2256,14 +2331,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:34:29</t>
+          <t>Última actualización: 08:53:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2447,37 +2522,37 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:53:40</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>09:28</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2486,7 +2561,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2502,43 +2577,143 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10:18</t>
+          <t>09:28</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>08:53:40</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>84</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>08:34:29</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>104</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:53:40</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>96</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:34:29</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D18" t="n">
         <v>116</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>08:53:40</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>109</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4369
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:53:40</t>
+          <t>Última actualización: 09:17:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 59</t>
+          <t>Total filas: 67</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:23</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,12 +1598,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:23</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>31</v>
+        <v>81</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,21 +1698,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>61</v>
+        <v>27</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,12 +1723,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>81</v>
+        <v>37</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>116</v>
+        <v>81</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>68</v>
+        <v>116</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>91</v>
+        <v>58</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:24</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>93</v>
+        <v>67</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,23 +1923,223 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>77</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>09:17:48</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>10:39</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>82</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>09:17:48</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D64" t="n">
+      <c r="D66" t="n">
+        <v>87</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>09:17:48</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>94</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>09:17:48</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>98</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>09:17:48</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>99</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>09:17:48</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>107</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>09:17:48</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
         <v>111</v>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>09:17:48</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>118</v>
+      </c>
+      <c r="E72" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1969,7 +2169,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:53:40</t>
+          <t>Última actualización: 09:17:48</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2460,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2274,7 +2474,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2331,7 +2531,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:53:40</t>
+          <t>Última actualización: 09:17:48</t>
         </is>
       </c>
     </row>
@@ -2547,7 +2747,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2561,7 +2761,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2597,7 +2797,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2611,7 +2811,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>84</v>
+        <v>60</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2647,7 +2847,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2661,7 +2861,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2697,7 +2897,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>08:53:40</t>
+          <t>09:17:48</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2711,7 +2911,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>109</v>
+        <v>85</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4370
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:17:48</t>
+          <t>Última actualización: 10:08:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 67</t>
+          <t>Total filas: 77</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>09:17:48</t>
+          <t>10:08:31</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>09:17:48</t>
+          <t>10:08:31</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>67</v>
+        <v>16</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>09:17:48</t>
+          <t>10:08:31</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>77</v>
+        <v>26</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>09:17:48</t>
+          <t>10:08:31</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>87</v>
+        <v>36</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>09:17:48</t>
+          <t>10:08:31</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>94</v>
+        <v>43</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>09:17:48</t>
+          <t>10:08:31</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>98</v>
+        <v>47</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>09:17:48</t>
+          <t>10:08:31</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>99</v>
+        <v>48</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>09:17:48</t>
+          <t>10:08:31</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>107</v>
+        <v>53</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>09:17:48</t>
+          <t>10:08:31</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>111</v>
+        <v>56</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,23 +2123,273 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>60</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>11:14</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>66</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>09:17:48</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D72" t="n">
+      <c r="D74" t="n">
         <v>118</v>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>76</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>11:31</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>83</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>87</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>93</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>96</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>106</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>107</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>116</v>
+      </c>
+      <c r="E82" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2156,7 +2406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2169,14 +2419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:17:48</t>
+          <t>Última actualización: 10:08:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2502,6 +2752,56 @@
         <v>81</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>87</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>96</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2518,7 +2818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2531,14 +2831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:17:48</t>
+          <t>Última actualización: 10:08:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -2822,7 +3122,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>10:08:31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2836,7 +3136,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>104</v>
+        <v>10</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2872,7 +3172,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>10:08:31</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2886,7 +3186,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>116</v>
+        <v>22</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2916,6 +3216,56 @@
       <c r="E19" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>35</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:08:31</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>75</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4371
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:08:31</t>
+          <t>Última actualización: 10:49:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 77</t>
+          <t>Total filas: 84</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2112,7 +2112,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>56</v>
+        <v>15</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,7 +2123,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>09:17:48</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>118</v>
+        <v>26</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>76</v>
+        <v>35</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2248,12 +2248,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2278,16 +2278,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>11:41</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>96</v>
+        <v>47</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>106</v>
+        <v>52</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>107</v>
+        <v>55</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,23 +2373,198 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>65</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>10:49:40</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>66</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>10:49:40</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
           <t>12:04</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D82" t="n">
-        <v>116</v>
-      </c>
-      <c r="E82" t="inlineStr">
+      <c r="D84" t="n">
+        <v>75</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>10:49:40</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>86</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>10:49:40</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>95</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>10:49:40</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>105</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>10:49:40</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>107</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>10:49:40</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>115</v>
+      </c>
+      <c r="E89" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2406,7 +2581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2419,14 +2594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:08:31</t>
+          <t>Última actualización: 10:49:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2760,12 +2935,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2774,7 +2949,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2790,18 +2965,43 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>87</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:49:40</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>11:44</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>96</v>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="D20" t="n">
+        <v>55</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2818,7 +3018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2831,14 +3031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:08:31</t>
+          <t>Última actualización: 10:49:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3247,23 +3447,48 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>10:49:40</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:22</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>33</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>10:08:31</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>11:23</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D22" t="n">
         <v>75</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4372
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:49:40</t>
+          <t>Última actualización: 11:12:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 84</t>
+          <t>Total filas: 90</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2312,7 +2312,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:54</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>66</v>
+        <v>42</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>75</v>
+        <v>43</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>95</v>
+        <v>63</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2503,16 +2503,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>107</v>
+        <v>73</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,23 +2548,173 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>78</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>11:12:15</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>82</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>11:12:15</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>84</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>11:12:15</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
           <t>12:44</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D89" t="n">
-        <v>115</v>
-      </c>
-      <c r="E89" t="inlineStr">
+      <c r="D92" t="n">
+        <v>92</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>11:12:15</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>94</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>11:12:15</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>103</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>11:12:15</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>113</v>
+      </c>
+      <c r="E95" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2581,7 +2731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2594,14 +2744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:49:40</t>
+          <t>Última actualización: 11:12:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -2960,7 +3110,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2974,7 +3124,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3002,6 +3152,56 @@
         <v>55</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>11:12:15</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>33</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:12:15</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>103</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3031,7 +3231,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:49:40</t>
+          <t>Última actualización: 11:12:15</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3672,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10:08:31</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3486,7 +3686,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4373
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:12:15</t>
+          <t>Última actualización: 11:45:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 90</t>
+          <t>Total filas: 97</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2412,7 +2412,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>42</v>
+        <v>9</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>95</v>
+        <v>30</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>73</v>
+        <v>38</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>10:49:40</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2603,16 +2603,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2678,16 +2678,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,23 +2698,198 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>59</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>61</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>70</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
           <t>13:05</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C98" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D95" t="n">
-        <v>113</v>
-      </c>
-      <c r="E95" t="inlineStr">
+      <c r="D98" t="n">
+        <v>80</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>90</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>97</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>99</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>107</v>
+      </c>
+      <c r="E102" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2731,7 +2906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2744,14 +2919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:12:15</t>
+          <t>Última actualización: 11:45:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -2935,7 +3110,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2945,11 +3120,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2960,7 +3135,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2970,11 +3145,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -3160,7 +3335,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3174,7 +3349,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3185,7 +3360,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3199,9 +3374,34 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>107</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3218,7 +3418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3231,14 +3431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:12:15</t>
+          <t>Última actualización: 11:45:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3689,6 +3889,31 @@
         <v>11</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>98</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4374
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E102"/>
+  <dimension ref="A1:E116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:45:05</t>
+          <t>Última actualización: 12:01:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 97</t>
+          <t>Total filas: 111</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2473,12 +2473,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2503,16 +2503,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>10:49:40</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>95</v>
+        <v>13</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2578,16 +2578,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2628,16 +2628,16 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>84</v>
+        <v>40</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2753,16 +2753,16 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2853,16 +2853,16 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,23 +2873,373 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
+          <t>12:01:57</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>45</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>12:01:57</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>53</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
           <t>11:45:05</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>70</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>12:01:57</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>63</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>80</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>12:01:57</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>73</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>90</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>12:01:57</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>80</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>97</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>12:01:57</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>82</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>99</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>12:01:57</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>90</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
         <is>
           <t>13:32</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C114" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D102" t="n">
+      <c r="D114" t="n">
         <v>107</v>
       </c>
-      <c r="E102" t="inlineStr">
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>12:01:57</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>103</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>12:01:57</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>113</v>
+      </c>
+      <c r="E116" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2906,7 +3256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2919,14 +3269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:45:05</t>
+          <t>Última actualización: 12:01:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -3360,12 +3710,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3374,7 +3724,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3390,18 +3740,68 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>70</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>12:01:57</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>90</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>13:32</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D25" t="n">
         <v>107</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3418,7 +3818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3431,14 +3831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:45:05</t>
+          <t>Última actualización: 12:01:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -3897,25 +4297,75 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>12:01:57</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>81</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>11:45:05</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>13:23</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D24" t="n">
         <v>98</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>12:01:57</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>108</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4375
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E116"/>
+  <dimension ref="A1:E126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:01:57</t>
+          <t>Última actualización: 12:33:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 111</t>
+          <t>Total filas: 121</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:12:15</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>11:12:15</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,12 +2848,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2862,7 +2862,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2903,16 +2903,16 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:46</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,12 +2923,12 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>80</v>
+        <v>22</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3028,16 +3028,16 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3053,16 +3053,16 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>82</v>
+        <v>48</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3128,16 +3128,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3153,16 +3153,16 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>107</v>
+        <v>51</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>103</v>
+        <v>58</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,23 +3223,273 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
+          <t>11:45:05</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>107</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>12:33:25</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>71</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
           <t>12:01:57</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
+      <c r="B118" t="inlineStr">
         <is>
           <t>13:54</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
+      <c r="C118" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D116" t="n">
+      <c r="D118" t="n">
         <v>113</v>
       </c>
-      <c r="E116" t="inlineStr">
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>12:33:25</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>82</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>12:33:25</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>91</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>12:33:25</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>98</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>12:33:25</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>101</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>12:33:25</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>101</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>12:33:25</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>101</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>12:33:25</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>111</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>12:33:25</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>118</v>
+      </c>
+      <c r="E126" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3269,7 +3519,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:01:57</t>
+          <t>Última actualización: 12:33:25</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3749,7 +3999,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>70</v>
+        <v>22</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3760,7 +4010,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3774,7 +4024,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -3818,7 +4068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3831,14 +4081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:01:57</t>
+          <t>Última actualización: 12:33:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4572,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4336,7 +4586,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4364,6 +4614,31 @@
         <v>108</v>
       </c>
       <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>12:33:25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>77</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4376
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E126"/>
+  <dimension ref="A1:E132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:33:25</t>
+          <t>Última actualización: 12:53:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 121</t>
+          <t>Total filas: 127</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -2923,12 +2923,12 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:53</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,12 +2948,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2962,7 +2962,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3003,16 +3003,16 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,12 +3023,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>80</v>
+        <v>11</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,12 +3073,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,12 +3123,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -3137,7 +3137,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,12 +3173,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -3187,7 +3187,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,12 +3223,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>107</v>
+        <v>38</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>13:54</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>113</v>
+        <v>51</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,12 +3298,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:54</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>82</v>
+        <v>113</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>91</v>
+        <v>62</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>98</v>
+        <v>63</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3453,16 +3453,16 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,23 +3473,173 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>81</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>12:53:36</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>81</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>12:53:36</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>83</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>12:53:36</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>91</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>12:53:36</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
           <t>14:31</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
+      <c r="C130" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D126" t="n">
-        <v>118</v>
-      </c>
-      <c r="E126" t="inlineStr">
+      <c r="D130" t="n">
+        <v>98</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>12:53:36</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>101</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>12:53:36</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>111</v>
+      </c>
+      <c r="E132" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3506,7 +3656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3519,14 +3669,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:33:25</t>
+          <t>Última actualización: 12:53:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -3960,12 +4110,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:53</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3974,7 +4124,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3985,12 +4135,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:01:57</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3999,7 +4149,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4015,16 +4165,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4035,23 +4185,73 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>12:53:36</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>38</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>11:45:05</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>13:32</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D26" t="n">
         <v>107</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>12:53:36</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>101</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4068,7 +4268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4081,14 +4281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:33:25</t>
+          <t>Última actualización: 12:53:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4547,7 +4747,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4561,7 +4761,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>81</v>
+        <v>29</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4622,7 +4822,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4636,11 +4836,36 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>12:53:36</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>109</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4377
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E132"/>
+  <dimension ref="A1:E140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:53:36</t>
+          <t>Última actualización: 13:12:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 127</t>
+          <t>Total filas: 135</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>13:12</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,12 +3098,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -3112,7 +3112,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3128,16 +3128,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,12 +3148,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -3162,7 +3162,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>97</v>
+        <v>9</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,12 +3198,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3228,16 +3228,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,12 +3248,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:45:05</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>107</v>
+        <v>19</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>11:45:05</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>51</v>
+        <v>107</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>13:54</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>113</v>
+        <v>32</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,12 +3323,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:54</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3353,16 +3353,16 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3428,16 +3428,16 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,12 +3448,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3462,7 +3462,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3478,16 +3478,16 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>83</v>
+        <v>61</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3578,16 +3578,16 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3603,16 +3603,16 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,23 +3623,223 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
+          <t>13:12:58</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>64</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>13:12:58</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>72</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
           <t>12:53:36</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr">
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>98</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>13:12:58</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>82</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>13:12:58</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>91</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>12:53:36</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
         <is>
           <t>14:44</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr">
+      <c r="C137" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D132" t="n">
+      <c r="D137" t="n">
         <v>111</v>
       </c>
-      <c r="E132" t="inlineStr">
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>13:12:58</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>102</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>13:12:58</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>109</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>13:12:58</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>112</v>
+      </c>
+      <c r="E140" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3656,7 +3856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3669,14 +3869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:53:36</t>
+          <t>Última actualización: 13:12:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4385,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4199,7 +4399,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4235,7 +4435,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4249,9 +4449,59 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:12:58</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>102</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:12:58</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>112</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4281,7 +4531,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:53:36</t>
+          <t>Última actualización: 13:12:58</t>
         </is>
       </c>
     </row>
@@ -4747,7 +4997,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4761,7 +5011,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4797,7 +5047,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:01:57</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4811,7 +5061,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>108</v>
+        <v>37</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4847,7 +5097,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4861,7 +5111,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4378
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E140"/>
+  <dimension ref="A1:E149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:12:58</t>
+          <t>Última actualización: 13:45:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 135</t>
+          <t>Total filas: 144</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>13:54</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,12 +3348,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:54</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3362,7 +3362,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>51</v>
+        <v>11</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,12 +3423,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>75</v>
+        <v>19</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:06</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>78</v>
+        <v>21</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>14:13</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>14:13</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>101</v>
+        <v>61</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:12:58</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>81</v>
+        <v>29</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>111</v>
+        <v>48</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3778,16 +3778,16 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>109</v>
+        <v>50</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3828,18 +3828,243 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>91</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>59</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>13:12:58</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>102</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>70</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>13:12:58</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>109</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>15:03</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>78</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
           <t>15:04</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
+      <c r="C146" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D140" t="n">
-        <v>112</v>
-      </c>
-      <c r="E140" t="inlineStr">
+      <c r="D146" t="n">
+        <v>79</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>90</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>99</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>110</v>
+      </c>
+      <c r="E149" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3856,7 +4081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3869,14 +4094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:12:58</t>
+          <t>Última actualización: 13:45:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -4460,21 +4685,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>102</v>
+        <v>50</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4490,18 +4715,93 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>102</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>70</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>15:04</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>112</v>
-      </c>
-      <c r="E29" t="inlineStr">
+      <c r="D31" t="n">
+        <v>79</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>110</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4518,7 +4818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4531,14 +4831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:12:58</t>
+          <t>Última actualización: 13:45:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -5072,7 +5372,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5086,7 +5386,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>57</v>
+        <v>5</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -5097,7 +5397,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5111,11 +5411,36 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>90</v>
+        <v>57</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>98</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4379
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E149"/>
+  <dimension ref="A1:E159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:45:34</t>
+          <t>Última actualización: 14:03:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 144</t>
+          <t>Total filas: 154</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3478,16 +3478,16 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>14:06</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,12 +3498,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>14:06</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3512,7 +3512,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>26</v>
+        <v>75</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>14:13</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,12 +3598,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:53:36</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>98</v>
+        <v>21</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:29</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>12:53:36</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3803,16 +3803,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>91</v>
+        <v>31</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3853,16 +3853,16 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:36</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>102</v>
+        <v>33</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>109</v>
+        <v>59</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>15:03</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3978,16 +3978,16 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4028,16 +4028,16 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,23 +4048,273 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
+          <t>14:03:57</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>61</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>14:03:57</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>63</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>14:03:57</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>15:14</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>71</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
           <t>13:45:34</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>90</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>14:03:57</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>80</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>99</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>14:03:57</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>91</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
         <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
+      <c r="C156" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D149" t="n">
+      <c r="D156" t="n">
         <v>110</v>
       </c>
-      <c r="E149" t="inlineStr">
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>14:03:57</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>101</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>14:03:57</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>111</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>14:03:57</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>16:01</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>118</v>
+      </c>
+      <c r="E159" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4081,7 +4331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4094,14 +4344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:45:34</t>
+          <t>Última actualización: 14:03:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -4660,7 +4910,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4674,7 +4924,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>82</v>
+        <v>31</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4710,7 +4960,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:12:58</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4724,7 +4974,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -4760,7 +5010,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4774,7 +5024,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -4785,23 +5035,48 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>14:03:57</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>91</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>13:45:34</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D32" t="n">
+      <c r="D33" t="n">
         <v>110</v>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4818,7 +5093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4831,14 +5106,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:45:34</t>
+          <t>Última actualización: 14:03:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -5397,7 +5672,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5411,7 +5686,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5422,25 +5697,75 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>14:03:57</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>79</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>13:45:34</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>15:23</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D29" t="n">
         <v>98</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>14:03:57</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>119</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4380
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E159"/>
+  <dimension ref="A1:E170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:03:57</t>
+          <t>Última actualización: 14:36:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 154</t>
+          <t>Total filas: 165</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3903,16 +3903,16 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:36</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:37</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>51</v>
+        <v>7</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>58</v>
+        <v>8</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>15:03</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>78</v>
+        <v>18</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>15:14</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>71</v>
+        <v>26</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4128,16 +4128,16 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>80</v>
+        <v>28</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4203,16 +4203,16 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:14</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>110</v>
+        <v>39</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4253,16 +4253,16 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>111</v>
+        <v>48</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,23 +4298,298 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
+          <t>14:36:54</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>58</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>13:45:34</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>110</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>14:36:54</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>68</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>14:36:54</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>15:50</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>74</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
           <t>14:03:57</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr">
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>111</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>14:36:54</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>79</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>14:03:57</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
         <is>
           <t>16:01</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
+      <c r="C165" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D159" t="n">
+      <c r="D165" t="n">
         <v>118</v>
       </c>
-      <c r="E159" t="inlineStr">
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>14:36:54</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>88</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>14:36:54</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>98</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>14:36:54</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>108</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>14:36:54</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>118</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>14:36:54</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>119</v>
+      </c>
+      <c r="E170" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4331,7 +4606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4344,14 +4619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:03:57</t>
+          <t>Última actualización: 14:36:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -4960,21 +5235,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:36</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -4985,12 +5260,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -4999,7 +5274,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>70</v>
+        <v>18</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5010,21 +5285,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -5035,21 +5310,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5060,23 +5335,48 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>14:36:54</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>58</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>13:45:34</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D34" t="n">
         <v>110</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5093,7 +5393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5106,14 +5406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:03:57</t>
+          <t>Última actualización: 14:36:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -5672,7 +5972,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5686,7 +5986,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5697,7 +5997,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5711,7 +6011,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5747,7 +6047,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5761,11 +6061,36 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>119</v>
+        <v>86</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>14:36:54</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>113</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4381
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E170"/>
+  <dimension ref="A1:E176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:36:54</t>
+          <t>Última actualización: 14:58:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 165</t>
+          <t>Total filas: 171</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4073,12 +4073,12 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:58</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -4087,7 +4087,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>15:02</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -4112,7 +4112,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,12 +4123,12 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>15:03</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>78</v>
+        <v>26</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>15:14</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>71</v>
+        <v>8</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,12 +4223,12 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:14</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>80</v>
+        <v>17</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,12 +4273,12 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>110</v>
+        <v>26</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>74</v>
+        <v>110</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>111</v>
+        <v>43</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>16:01</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>98</v>
+        <v>57</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>108</v>
+        <v>58</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,17 +4548,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -4573,23 +4573,173 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>66</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>14:58:46</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>76</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>14:58:46</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>86</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>14:58:46</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>96</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>14:58:46</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
           <t>16:35</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr">
+      <c r="C174" t="inlineStr">
         <is>
           <t>83_ALUAR</t>
         </is>
       </c>
-      <c r="D170" t="n">
-        <v>119</v>
-      </c>
-      <c r="E170" t="inlineStr">
+      <c r="D174" t="n">
+        <v>97</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>14:58:46</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>106</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>14:58:46</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>117</v>
+      </c>
+      <c r="E176" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4619,7 +4769,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:36:54</t>
+          <t>Última actualización: 14:58:46</t>
         </is>
       </c>
     </row>
@@ -5310,7 +5460,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5324,7 +5474,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5335,7 +5485,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5349,7 +5499,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5406,7 +5556,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:36:54</t>
+          <t>Última actualización: 14:58:46</t>
         </is>
       </c>
     </row>
@@ -5997,7 +6147,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -6011,7 +6161,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -6047,7 +6197,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6061,7 +6211,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -6072,7 +6222,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:58:46</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -6086,7 +6236,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>113</v>
+        <v>91</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4382
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E176"/>
+  <dimension ref="A1:E183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:58:46</t>
+          <t>Última actualización: 15:34:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 171</t>
+          <t>Total filas: 178</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4387,7 +4387,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>110</v>
+        <v>1</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>14:58:46</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>111</v>
+        <v>17</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,12 +4498,12 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>14:58:46</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>57</v>
+        <v>111</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>14:58:46</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>16:01</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>118</v>
+        <v>22</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,12 +4573,12 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:58:46</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>66</v>
+        <v>118</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:58:46</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>14:58:46</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>14:58:46</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:16</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>14:58:46</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>97</v>
+        <v>50</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>14:58:46</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>106</v>
+        <v>60</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,23 +4723,198 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>14:58:46</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>61</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>15:34:27</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>70</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>15:34:27</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>16:52</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>78</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>15:34:27</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
           <t>16:55</t>
         </is>
       </c>
-      <c r="C176" t="inlineStr">
+      <c r="C179" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D176" t="n">
+      <c r="D179" t="n">
+        <v>81</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>15:34:27</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>90</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>15:34:27</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>101</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>15:34:27</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>110</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>15:34:27</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
         <v>117</v>
       </c>
-      <c r="E176" t="inlineStr">
+      <c r="E183" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4756,7 +4931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4769,14 +4944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:58:46</t>
+          <t>Última actualización: 15:34:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -5510,7 +5685,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5524,9 +5699,34 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>110</v>
+        <v>1</v>
       </c>
       <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>15:34:27</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>101</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5543,7 +5743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5556,14 +5756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:58:46</t>
+          <t>Última actualización: 15:34:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -6222,25 +6422,100 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>15:34:27</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>29</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>14:58:46</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>16:29</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D32" t="n">
         <v>91</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>15:34:27</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>56</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>15:34:27</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>109</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4383
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E183"/>
+  <dimension ref="A1:E194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:34:27</t>
+          <t>Última actualización: 16:09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 178</t>
+          <t>Total filas: 189</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:21</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4703,16 +4703,16 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>61</v>
+        <v>16</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>16:52</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>78</v>
+        <v>26</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:42</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>81</v>
+        <v>33</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>90</v>
+        <v>35</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>101</v>
+        <v>42</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4878,16 +4878,16 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>16:52</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,23 +4898,298 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>46</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
           <t>15:34:27</t>
         </is>
       </c>
-      <c r="B183" t="inlineStr">
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>90</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>56</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>66</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>75</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>15:34:27</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
         <is>
           <t>17:31</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr">
+      <c r="C188" t="inlineStr">
         <is>
           <t>23_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D183" t="n">
+      <c r="D188" t="n">
         <v>117</v>
       </c>
-      <c r="E183" t="inlineStr">
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>82</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>84</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>86</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>96</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>106</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>115</v>
+      </c>
+      <c r="E194" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4931,7 +5206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4944,14 +5219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:34:27</t>
+          <t>Última actualización: 16:09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -5710,7 +5985,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5724,9 +5999,59 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>101</v>
+        <v>66</v>
       </c>
       <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>96</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>106</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5756,7 +6081,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:34:27</t>
+          <t>Última actualización: 16:09:00</t>
         </is>
       </c>
     </row>
@@ -6472,7 +6797,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6486,7 +6811,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6497,7 +6822,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6511,7 +6836,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4384
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E194"/>
+  <dimension ref="A1:E203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:00</t>
+          <t>Última actualización: 16:36:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 189</t>
+          <t>Total filas: 198</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>16:42</t>
+          <t>16:36</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4853,16 +4853,16 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:42</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>16:52</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>78</v>
+        <v>8</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4928,16 +4928,16 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>16:52</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5003,16 +5003,16 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>117</v>
+        <v>39</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>82</v>
+        <v>48</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:28</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>15:34:27</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5153,16 +5153,16 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5178,18 +5178,243 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>84</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>16:36:26</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>59</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>16:36:26</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>60</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>16:36:26</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>68</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>16:09:00</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>96</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>16:36:26</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>79</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>16:36:26</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
           <t>18:04</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr">
+      <c r="C200" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D194" t="n">
-        <v>115</v>
-      </c>
-      <c r="E194" t="inlineStr">
+      <c r="D200" t="n">
+        <v>88</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>16:36:26</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>99</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>16:36:26</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>108</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>16:36:26</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>118</v>
+      </c>
+      <c r="E203" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5206,7 +5431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5219,14 +5444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:00</t>
+          <t>Última actualización: 16:36:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -5985,7 +6210,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5999,7 +6224,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>66</v>
+        <v>39</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6010,12 +6235,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -6024,7 +6249,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6040,18 +6265,68 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>96</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>16:36:26</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>17:55</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>106</v>
-      </c>
-      <c r="E37" t="inlineStr">
+      <c r="D38" t="n">
+        <v>79</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>16:36:26</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>99</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6068,7 +6343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6081,14 +6356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:00</t>
+          <t>Última actualización: 16:36:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6822,23 +7097,48 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>15</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>16:36:26</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>17:23</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>74</v>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="D35" t="n">
+        <v>47</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4385
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E203"/>
+  <dimension ref="A1:E208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:36:26</t>
+          <t>Última actualización: 16:54:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 198</t>
+          <t>Total filas: 203</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4962,7 +4962,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>56</v>
+        <v>11</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5062,7 +5062,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>15:34:27</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>117</v>
+        <v>82</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,12 +5273,12 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -5287,7 +5287,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>79</v>
+        <v>51</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,23 +5398,148 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
+          <t>16:54:18</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>88</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
           <t>16:36:26</t>
         </is>
       </c>
-      <c r="B203" t="inlineStr">
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>108</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>16:54:18</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>91</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>16:54:18</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
         <is>
           <t>18:34</t>
         </is>
       </c>
-      <c r="C203" t="inlineStr">
+      <c r="C206" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D203" t="n">
-        <v>118</v>
-      </c>
-      <c r="E203" t="inlineStr">
+      <c r="D206" t="n">
+        <v>100</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>16:54:18</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>102</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>16:54:18</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>110</v>
+      </c>
+      <c r="E208" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5444,7 +5569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:36:26</t>
+          <t>Última actualización: 16:54:18</t>
         </is>
       </c>
     </row>
@@ -6210,7 +6335,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6224,7 +6349,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6260,7 +6385,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6274,7 +6399,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6285,7 +6410,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6299,7 +6424,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6310,7 +6435,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6324,7 +6449,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6343,7 +6468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6356,14 +6481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:36:26</t>
+          <t>Última actualización: 16:54:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -7122,23 +7247,73 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>14</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>16:54:18</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>17:23</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>47</v>
-      </c>
-      <c r="E35" t="inlineStr">
+      <c r="D36" t="n">
+        <v>29</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16:54:18</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>111</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4386
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E208"/>
+  <dimension ref="A1:E216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:54:18</t>
+          <t>Última actualización: 17:12:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 203</t>
+          <t>Total filas: 211</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -5023,12 +5023,12 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5053,16 +5053,16 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>17:26</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>17:28</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>52</v>
+        <v>14</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:36:26</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:28</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>82</v>
+        <v>52</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5178,16 +5178,16 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>41</v>
+        <v>84</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,12 +5248,12 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5353,16 +5353,16 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5403,16 +5403,16 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>108</v>
+        <v>52</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>91</v>
+        <v>62</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5478,16 +5478,16 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5503,16 +5503,16 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,23 +5523,223 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>71</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>72</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
           <t>16:54:18</t>
         </is>
       </c>
-      <c r="B208" t="inlineStr">
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>91</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>82</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>84</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
         <is>
           <t>18:44</t>
         </is>
       </c>
-      <c r="C208" t="inlineStr">
+      <c r="C213" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D208" t="n">
-        <v>110</v>
-      </c>
-      <c r="E208" t="inlineStr">
+      <c r="D213" t="n">
+        <v>92</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>102</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>107</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>112</v>
+      </c>
+      <c r="E216" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5556,7 +5756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5569,14 +5769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:54:18</t>
+          <t>Última actualización: 17:12:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -6335,12 +6535,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -6349,7 +6549,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6360,21 +6560,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:36:26</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6385,12 +6585,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -6399,7 +6599,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6415,16 +6615,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6435,23 +6635,123 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>42</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>16:54:18</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>61</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>62</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>16:54:18</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
         <is>
           <t>18:15</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D42" t="n">
         <v>81</v>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>107</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6468,7 +6768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6481,14 +6781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:54:18</t>
+          <t>Última actualización: 17:12:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -7272,48 +7572,123 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>10</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>16:54:18</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>29</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>92</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>16:54:18</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
         <is>
           <t>18:45</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D40" t="n">
         <v>111</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4387
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E216"/>
+  <dimension ref="A1:E226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:12:40</t>
+          <t>Última actualización: 17:44:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 211</t>
+          <t>Total filas: 221</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>17:12:40</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>17:12:40</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>18:14</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:07</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>81</v>
+        <v>23</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:12:40</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>88</v>
+        <v>62</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>17:12:40</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>17:12:40</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5578,16 +5578,16 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5603,16 +5603,16 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5628,16 +5628,16 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>17:12:40</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>92</v>
+        <v>41</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>17:12:40</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>102</v>
+        <v>50</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>17:12:40</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>18:59</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>107</v>
+        <v>52</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,23 +5723,273 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
+          <t>17:44:09</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>60</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>17:44:09</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>70</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
           <t>17:12:40</t>
         </is>
       </c>
-      <c r="B216" t="inlineStr">
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>107</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>17:44:09</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>76</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>17:12:40</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
         <is>
           <t>19:04</t>
         </is>
       </c>
-      <c r="C216" t="inlineStr">
+      <c r="C220" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D216" t="n">
+      <c r="D220" t="n">
         <v>112</v>
       </c>
-      <c r="E216" t="inlineStr">
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>17:44:09</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>81</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>17:44:09</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>92</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>17:44:09</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>93</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>17:44:09</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>97</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>17:44:09</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>100</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>17:44:09</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>101</v>
+      </c>
+      <c r="E226" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5756,7 +6006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5769,14 +6019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:12:40</t>
+          <t>Última actualización: 17:44:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -6610,7 +6860,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6624,7 +6874,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6660,7 +6910,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6674,7 +6924,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -6710,7 +6960,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -6724,7 +6974,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>81</v>
+        <v>31</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -6752,6 +7002,56 @@
         <v>107</v>
       </c>
       <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>17:44:09</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>76</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>17:44:09</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>101</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6768,7 +7068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6781,14 +7081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:12:40</t>
+          <t>Última actualización: 17:44:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -7672,7 +7972,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7686,11 +7986,36 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>111</v>
+        <v>61</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>17:44:09</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>91</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4388
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E226"/>
+  <dimension ref="A1:E229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:44:09</t>
+          <t>Última actualización: 18:03:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 221</t>
+          <t>Total filas: 224</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5462,7 +5462,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5537,7 +5537,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5662,7 +5662,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5687,7 +5687,7 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5712,7 +5712,7 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5737,7 +5737,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5762,7 +5762,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5848,7 +5848,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5887,7 +5887,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5948,7 +5948,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5987,9 +5987,84 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>18:03:05</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>19:27</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>84</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>18:03:05</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>106</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>18:03:05</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>107</v>
+      </c>
+      <c r="E229" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6019,7 +6094,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:44:09</t>
+          <t>Última actualización: 18:03:05</t>
         </is>
       </c>
     </row>
@@ -6960,7 +7035,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -6974,7 +7049,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7035,7 +7110,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7049,7 +7124,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -7068,7 +7143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7081,14 +7156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:44:09</t>
+          <t>Última actualización: 18:03:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -7972,7 +8047,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7986,7 +8061,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7997,7 +8072,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8011,11 +8086,36 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>18:03:05</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>104</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4389
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E229"/>
+  <dimension ref="A1:E234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:03:05</t>
+          <t>Última actualización: 18:34:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 224</t>
+          <t>Total filas: 229</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5687,7 +5687,7 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5712,7 +5712,7 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5737,7 +5737,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5762,7 +5762,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>17:12:40</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5837,7 +5837,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>112</v>
+        <v>30</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5887,7 +5887,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>73</v>
+        <v>42</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,12 +5898,12 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>82</v>
+        <v>50</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>19:27</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>84</v>
+        <v>51</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6028,16 +6028,16 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:27</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>106</v>
+        <v>84</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,23 +6048,148 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
+          <t>19:29</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>55</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>18:34:28</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>75</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>18:34:28</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
           <t>19:50</t>
         </is>
       </c>
-      <c r="C229" t="inlineStr">
+      <c r="C231" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D229" t="n">
-        <v>107</v>
-      </c>
-      <c r="E229" t="inlineStr">
+      <c r="D231" t="n">
+        <v>76</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>18:34:28</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>91</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>18:34:28</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>101</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>18:34:28</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>101</v>
+      </c>
+      <c r="E234" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6081,7 +6206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6094,14 +6219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:03:05</t>
+          <t>Última actualización: 18:34:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -7085,7 +7210,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7099,7 +7224,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7110,7 +7235,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7124,9 +7249,34 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>82</v>
+        <v>51</v>
       </c>
       <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>18:34:28</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>101</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7156,7 +7306,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:03:05</t>
+          <t>Última actualización: 18:34:28</t>
         </is>
       </c>
     </row>
@@ -8047,7 +8197,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -8061,7 +8211,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -8072,7 +8222,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8086,7 +8236,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>72</v>
+        <v>41</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -8097,7 +8247,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8111,7 +8261,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>104</v>
+        <v>73</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4390
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E234"/>
+  <dimension ref="A1:E240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:34:28</t>
+          <t>Última actualización: 18:54:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 229</t>
+          <t>Total filas: 235</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5762,7 +5762,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5848,7 +5848,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5887,7 +5887,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5933,11 +5933,11 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>97</v>
+        <v>23</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>19:27</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,12 +6048,12 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>19:29</t>
+          <t>19:27</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -6062,7 +6062,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>55</v>
+        <v>84</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6078,16 +6078,16 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:29</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>91</v>
+        <v>56</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>101</v>
+        <v>62</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,23 +6173,173 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
+          <t>18:54:05</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>68</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
           <t>18:34:28</t>
         </is>
       </c>
-      <c r="B234" t="inlineStr">
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>91</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>18:34:28</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
         <is>
           <t>20:15</t>
         </is>
       </c>
-      <c r="C234" t="inlineStr">
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>101</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>18:54:05</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D234" t="n">
-        <v>101</v>
-      </c>
-      <c r="E234" t="inlineStr">
+      <c r="D237" t="n">
+        <v>81</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>18:54:05</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>82</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>18:54:05</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>106</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>18:54:05</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>107</v>
+      </c>
+      <c r="E240" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6206,7 +6356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6219,14 +6369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:34:28</t>
+          <t>Última actualización: 18:54:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -7210,7 +7360,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7224,7 +7374,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7235,7 +7385,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7249,7 +7399,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -7260,7 +7410,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7274,9 +7424,59 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>18:54:05</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>106</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>18:54:05</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>107</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7293,7 +7493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7306,14 +7506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:34:28</t>
+          <t>Última actualización: 18:54:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -8222,7 +8422,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8236,7 +8436,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -8247,7 +8447,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8261,9 +8461,34 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>18:54:05</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>108</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4391
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E240"/>
+  <dimension ref="A1:E247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:54:06</t>
+          <t>Última actualización: 19:11:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 235</t>
+          <t>Total filas: 242</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>42</v>
+        <v>5</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5928,16 +5928,16 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5958,7 +5958,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D225" t="n">
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>17:44:09</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>97</v>
+        <v>23</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>17:44:09</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>30</v>
+        <v>97</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>18:03:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>19:27</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>84</v>
+        <v>14</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,12 +6073,12 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:03:05</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>19:29</t>
+          <t>19:27</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>55</v>
+        <v>84</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,17 +6098,17 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:29</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D231" t="n">
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,12 +6198,12 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -6212,7 +6212,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>91</v>
+        <v>50</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>18:34:28</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>18:34:28</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6328,18 +6328,193 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>82</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>19:11:26</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>20:36</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>85</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>19:11:26</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>88</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>18:54:05</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>106</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>19:11:26</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C240" t="inlineStr">
+      <c r="C244" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D240" t="n">
-        <v>107</v>
-      </c>
-      <c r="E240" t="inlineStr">
+      <c r="D244" t="n">
+        <v>90</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>19:11:26</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>105</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>19:11:26</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>115</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>19:11:26</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>115</v>
+      </c>
+      <c r="E247" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6356,7 +6531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6369,14 +6544,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:54:06</t>
+          <t>Última actualización: 19:11:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -7385,7 +7560,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7399,7 +7574,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -7410,7 +7585,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7424,7 +7599,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -7435,12 +7610,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -7449,7 +7624,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -7465,18 +7640,68 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>106</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>19:11:26</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D48" t="n">
-        <v>107</v>
-      </c>
-      <c r="E48" t="inlineStr">
+      <c r="D49" t="n">
+        <v>90</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>19:11:26</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>115</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7493,7 +7718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7506,14 +7731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:54:06</t>
+          <t>Última actualización: 19:11:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -8422,7 +8647,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8436,7 +8661,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -8447,7 +8672,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8461,7 +8686,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8489,6 +8714,31 @@
         <v>108</v>
       </c>
       <c r="E43" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>19:11:26</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>94</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4392
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E247"/>
+  <dimension ref="A1:E251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:11:26</t>
+          <t>Última actualización: 19:41:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 242</t>
+          <t>Total filas: 246</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6137,7 +6137,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6162,7 +6162,7 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,7 +6173,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -6187,7 +6187,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6212,7 +6212,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6273,7 +6273,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6323,7 +6323,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -6337,7 +6337,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>82</v>
+        <v>35</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,7 +6348,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -6362,7 +6362,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6398,7 +6398,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -6412,7 +6412,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>106</v>
+        <v>59</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>115</v>
+        <v>76</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,23 +6498,123 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>81</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>19:41:17</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
           <t>21:06</t>
         </is>
       </c>
-      <c r="C247" t="inlineStr">
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>85</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>19:41:17</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D247" t="n">
-        <v>115</v>
-      </c>
-      <c r="E247" t="inlineStr">
+      <c r="D249" t="n">
+        <v>85</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>19:41:17</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>113</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>19:41:17</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>116</v>
+      </c>
+      <c r="E251" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6544,7 +6644,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:11:26</t>
+          <t>Última actualización: 19:41:17</t>
         </is>
       </c>
     </row>
@@ -7585,7 +7685,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7599,7 +7699,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -7635,7 +7735,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7649,7 +7749,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>106</v>
+        <v>59</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -7660,7 +7760,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7674,7 +7774,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -7685,7 +7785,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7699,7 +7799,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -7718,7 +7818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7731,14 +7831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:11:26</t>
+          <t>Última actualización: 19:41:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -8672,7 +8772,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8686,7 +8786,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8697,12 +8797,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:41:17</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -8711,7 +8811,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>108</v>
+        <v>58</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8722,23 +8822,48 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>18:54:05</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>108</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>19:11:26</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D44" t="n">
+      <c r="D45" t="n">
         <v>94</v>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4393
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E251"/>
+  <dimension ref="A1:E257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:41:17</t>
+          <t>Última actualización: 20:05:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 246</t>
+          <t>Total filas: 252</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5933,11 +5933,11 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5958,7 +5958,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D225" t="n">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:08</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6308,11 +6308,11 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>64</v>
+        <v>10</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,12 +6323,12 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -6337,7 +6337,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6353,16 +6353,16 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>88</v>
+        <v>31</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,12 +6398,12 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -6412,7 +6412,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6428,16 +6428,16 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>105</v>
+        <v>36</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,12 +6473,12 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -6487,7 +6487,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>76</v>
+        <v>51</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6503,16 +6503,16 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6553,16 +6553,16 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>113</v>
+        <v>60</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6603,18 +6603,168 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>85</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>20:05:28</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>61</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>20:05:28</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>89</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>20:05:28</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>91</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>20:05:28</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
           <t>21:37</t>
         </is>
       </c>
-      <c r="C251" t="inlineStr">
+      <c r="C255" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D251" t="n">
-        <v>116</v>
-      </c>
-      <c r="E251" t="inlineStr">
+      <c r="D255" t="n">
+        <v>92</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>20:05:28</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>95</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>20:05:28</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>114</v>
+      </c>
+      <c r="E257" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6644,7 +6794,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:41:17</t>
+          <t>Última actualización: 20:05:28</t>
         </is>
       </c>
     </row>
@@ -7685,7 +7835,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7699,7 +7849,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -7710,7 +7860,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7724,7 +7874,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>88</v>
+        <v>34</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -7760,7 +7910,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7774,7 +7924,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -7785,7 +7935,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7799,7 +7949,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -7818,7 +7968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7831,14 +7981,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:41:17</t>
+          <t>Última actualización: 20:05:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -8797,7 +8947,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8811,7 +8961,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8864,6 +9014,31 @@
         <v>94</v>
       </c>
       <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>20:05:28</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>87</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4394
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E257"/>
+  <dimension ref="A1:E262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:05:28</t>
+          <t>Última actualización: 20:31:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 252</t>
+          <t>Total filas: 257</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5933,11 +5933,11 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5958,7 +5958,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D225" t="n">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6308,11 +6308,11 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>10</v>
+        <v>64</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,7 +6323,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -6333,11 +6333,11 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>64</v>
+        <v>10</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,12 +6423,12 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6478,16 +6478,16 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6528,16 +6528,16 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>81</v>
+        <v>26</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6578,16 +6578,16 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6603,16 +6603,16 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6628,16 +6628,16 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>89</v>
+        <v>35</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>91</v>
+        <v>35</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>92</v>
+        <v>63</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,21 +6723,21 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,23 +6748,148 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>66</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
           <t>20:05:28</t>
         </is>
       </c>
-      <c r="B257" t="inlineStr">
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>95</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>21:43</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>72</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
         <is>
           <t>21:59</t>
         </is>
       </c>
-      <c r="C257" t="inlineStr">
+      <c r="C260" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D257" t="n">
-        <v>114</v>
-      </c>
-      <c r="E257" t="inlineStr">
+      <c r="D260" t="n">
+        <v>88</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>96</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>115</v>
+      </c>
+      <c r="E262" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6781,7 +6906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6794,14 +6919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:05:28</t>
+          <t>Última actualización: 20:31:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -7860,21 +7985,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -7885,12 +8010,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>19:41:17</t>
+          <t>20:05:28</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -7899,7 +8024,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -7910,21 +8035,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -7940,18 +8065,43 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>36</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>21:06</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D50" t="n">
-        <v>61</v>
-      </c>
-      <c r="E50" t="inlineStr">
+      <c r="D51" t="n">
+        <v>35</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7968,7 +8118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7981,14 +8131,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:05:28</t>
+          <t>Última actualización: 20:31:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -8947,7 +9097,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8961,7 +9111,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -9022,7 +9172,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -9036,11 +9186,36 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>98</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4395
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E262"/>
+  <dimension ref="A1:E266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:31:19</t>
+          <t>Última actualización: 20:51:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 257</t>
+          <t>Total filas: 261</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5933,11 +5933,11 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -6537,7 +6537,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6637,7 +6637,7 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6673,7 +6673,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6687,7 +6687,7 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6712,7 +6712,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6737,7 +6737,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,7 +6748,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -6762,7 +6762,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6798,12 +6798,12 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>21:43</t>
+          <t>21:41</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -6812,7 +6812,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6828,16 +6828,16 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>21:59</t>
+          <t>21:43</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>22:07</t>
+          <t>21:59</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,23 +6873,123 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>76</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>20:51:31</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
           <t>22:26</t>
         </is>
       </c>
-      <c r="C262" t="inlineStr">
+      <c r="C263" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D262" t="n">
-        <v>115</v>
-      </c>
-      <c r="E262" t="inlineStr">
+      <c r="D263" t="n">
+        <v>95</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>20:51:31</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>22:35</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>104</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>20:51:31</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>106</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>20:51:31</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>22:41</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>110</v>
+      </c>
+      <c r="E266" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6906,7 +7006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6919,14 +7019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:31:19</t>
+          <t>Última actualización: 20:51:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -8085,7 +8185,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -8099,9 +8199,34 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>20:51:31</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>106</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8131,7 +8256,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:31:19</t>
+          <t>Última actualización: 20:51:31</t>
         </is>
       </c>
     </row>
@@ -9172,7 +9297,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -9186,7 +9311,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -9197,7 +9322,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -9211,7 +9336,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4396
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-17.xlsx
+++ b/data/horarios-141-2026-08-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E266"/>
+  <dimension ref="A1:E271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:51:31</t>
+          <t>Última actualización: 21:31:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 261</t>
+          <t>Total filas: 266</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:03:46</t>
+          <t>05:54:40</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,11 +908,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:54:40</t>
+          <t>07:03:46</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -933,11 +933,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:02:51</t>
+          <t>08:34:29</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:34:29</t>
+          <t>08:02:51</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:33:25</t>
+          <t>13:45:34</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>13:45:34</t>
+          <t>12:33:25</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>14:36:54</t>
+          <t>14:03:57</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:03:57</t>
+          <t>14:36:54</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>16:09:00</t>
+          <t>16:54:18</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>16:54:18</t>
+          <t>16:09:00</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>18:54:05</t>
+          <t>19:11:26</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>19:11:26</t>
+          <t>18:54:05</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5933,11 +5933,11 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -6698,12 +6698,12 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>20:51:31</t>
+          <t>21:31:34</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:33</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -6712,7 +6712,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6728,16 +6728,16 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,21 +6748,21 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>20:51:31</t>
+          <t>21:31:34</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>20:05:28</t>
+          <t>21:31:34</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>95</v>
+        <v>6</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,12 +6798,12 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>20:51:31</t>
+          <t>21:31:34</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>21:41</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -6812,7 +6812,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,12 +6823,12 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:51:31</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>21:43</t>
+          <t>21:41</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -6837,7 +6837,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>20:51:31</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>21:59</t>
+          <t>21:43</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,21 +6873,21 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>20:51:31</t>
+          <t>21:31:34</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>22:07</t>
+          <t>21:59</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>20:51:31</t>
+          <t>21:31:34</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>22:26</t>
+          <t>22:07</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>95</v>
+        <v>36</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>20:51:31</t>
+          <t>21:31:34</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>22:35</t>
+          <t>22:26</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>20:51:31</t>
+          <t>21:31:34</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>22:37</t>
+          <t>22:29</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>106</v>
+        <v>58</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,23 +6973,148 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>20:51:31</t>
+          <t>21:31:34</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
+          <t>22:35</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>64</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>21:31:34</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>66</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>21:31:34</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
           <t>22:41</t>
         </is>
       </c>
-      <c r="C266" t="inlineStr">
+      <c r="C268" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D266" t="n">
-        <v>110</v>
-      </c>
-      <c r="E266" t="inlineStr">
+      <c r="D268" t="n">
+        <v>70</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>21:31:34</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>22:55</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>84</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>21:31:34</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>23:07</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>96</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>21:31:34</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>23:28</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>117</v>
+      </c>
+      <c r="E271" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7006,7 +7131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7019,14 +7144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:51:31</t>
+          <t>Última actualización: 21:31:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 49</t>
         </is>
       </c>
     </row>
@@ -8210,23 +8335,73 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>20:51:31</t>
+          <t>21:31:34</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>22:29</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>58</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>21:31:34</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>22:37</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D52" t="n">
-        <v>106</v>
-      </c>
-      <c r="E52" t="inlineStr">
+      <c r="D53" t="n">
+        <v>66</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>21:31:34</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>23:28</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>117</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8243,7 +8418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8256,14 +8431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:51:31</t>
+          <t>Última actualización: 21:31:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -9297,12 +9472,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>20:51:31</t>
+          <t>21:31:34</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>21:32</t>
+          <t>21:31</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -9311,7 +9486,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -9327,18 +9502,43 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>41</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>21:31:34</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>22:09</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D47" t="n">
-        <v>78</v>
-      </c>
-      <c r="E47" t="inlineStr">
+      <c r="D48" t="n">
+        <v>38</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>